<commit_message>
数据更新 2026-08-11（GitHub Actions 自动）
模式：daily

═══ 数据状态 ═══
  指数: 2026-08-11 ✓
  ETF: 2026-08-11 ✓
  推荐20: 2026-08-11 ✓
  其他成份: 2026-08-11 ✓
  自选: 2026-08-11 ✓
  成分样本: 2026-08-10 ⚠️ 滞后 1 天
  回测: 2026-08-10 ⚠️ 已过期（维护→1 重跑，约1分钟）
  季度检测: 从未执行（深度更新或维护可执行）
  失败清单: 2 只（北交所无数据源，预期内）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="980092" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="980092" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'980092'!$A$1:$E$101</definedName>

</xml_diff>

<commit_message>
数据更新 2026-08-12（GitHub Actions 自动）
模式：daily

═══ 数据状态 ═══
  指数: 2026-08-12 ✓
  ETF: 2026-08-12 ✓
  推荐20: 2026-08-12 ✓
  其他成份: 2026-08-12 ✓
  自选: 2026-08-12 ✓
  成分样本: 2026-08-11 ⚠️ 滞后 1 天
  回测: 2026-08-10 ⚠️ 已过期（维护→1 重跑，约1分钟）
  季度检测: 从未执行（深度更新或维护可执行）
  失败清单: 2 只（北交所无数据源，预期内）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -489,21 +489,21 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>601728</t>
+          <t>600938</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>中国电信</t>
+          <t>中国海油</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>电信业务</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9.02</v>
+        <v>9.24</v>
       </c>
     </row>
     <row r="3">
@@ -512,21 +512,21 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>600938</t>
+          <t>601728</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>中国海油</t>
+          <t>中国电信</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>电信业务</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>8.779999999999999</v>
+        <v>9.09</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6.33</v>
+        <v>6.31</v>
       </c>
     </row>
     <row r="5">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5.58</v>
+        <v>5.55</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.28</v>
+        <v>5.19</v>
       </c>
     </row>
     <row r="7">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>4.35</v>
+        <v>4.25</v>
       </c>
     </row>
     <row r="8">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>4.02</v>
+        <v>4.13</v>
       </c>
     </row>
     <row r="9">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="10">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3.52</v>
+        <v>3.51</v>
       </c>
     </row>
     <row r="11">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3.3</v>
+        <v>3.27</v>
       </c>
     </row>
     <row r="12">
@@ -1219,17 +1219,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>600352</t>
+          <t>601880</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>浙江龙盛</t>
+          <t>辽港股份</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1244,17 +1244,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>601880</t>
+          <t>600352</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>辽港股份</t>
+          <t>浙江龙盛</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1269,17 +1269,17 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>600546</t>
+          <t>600398</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>山煤国际</t>
+          <t>海澜之家</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1294,17 +1294,17 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>600398</t>
+          <t>600546</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>海澜之家</t>
+          <t>山煤国际</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -1344,17 +1344,17 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>603444</t>
+          <t>600295</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>吉比特</t>
+          <t>鄂尔多斯</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -1369,17 +1369,17 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>600295</t>
+          <t>603444</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>鄂尔多斯</t>
+          <t>吉比特</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -1394,17 +1394,17 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>600320</t>
+          <t>600060</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>振华重工</t>
+          <t>海信视像</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -1419,17 +1419,17 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>600060</t>
+          <t>600320</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>海信视像</t>
+          <t>振华重工</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -1444,12 +1444,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>600380</t>
+          <t>603883</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>健康元</t>
+          <t>老百姓</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>603883</t>
+          <t>600380</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>老百姓</t>
+          <t>健康元</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1694,17 +1694,17 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>603766</t>
+          <t>002761</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>隆鑫通用</t>
+          <t>浙江建投</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -1719,17 +1719,17 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>002761</t>
+          <t>603766</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>浙江建投</t>
+          <t>隆鑫通用</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -1794,17 +1794,17 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>002545</t>
+          <t>600729</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>东方铁塔</t>
+          <t>重百集团</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -1819,17 +1819,17 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>600729</t>
+          <t>002039</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>重百集团</t>
+          <t>黔源电力</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -1844,17 +1844,17 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>002039</t>
+          <t>002545</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>黔源电力</t>
+          <t>东方铁塔</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -1894,17 +1894,17 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>600004</t>
+          <t>002727</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>白云机场</t>
+          <t>一心堂</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -1919,17 +1919,17 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>000957</t>
+          <t>600004</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>中通客车</t>
+          <t>白云机场</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -1969,12 +1969,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>000719</t>
+          <t>002416</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>中原传媒</t>
+          <t>爱施德</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -1994,17 +1994,17 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>002727</t>
+          <t>000957</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>一心堂</t>
+          <t>中通客车</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -2019,12 +2019,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>002416</t>
+          <t>000719</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>爱施德</t>
+          <t>中原传媒</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -2219,17 +2219,17 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>301039</t>
+          <t>000597</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>中集车辆</t>
+          <t>东北制药</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -2244,17 +2244,17 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>000597</t>
+          <t>301039</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>东北制药</t>
+          <t>中集车辆</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -2744,17 +2744,17 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>002478</t>
+          <t>300389</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>常宝股份</t>
+          <t>艾比森</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -2769,17 +2769,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>300389</t>
+          <t>002478</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>艾比森</t>
+          <t>常宝股份</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -2794,17 +2794,17 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>300228</t>
+          <t>000026</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>富瑞特装</t>
+          <t>飞亚达</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -2819,17 +2819,17 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>000026</t>
+          <t>300228</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>飞亚达</t>
+          <t>富瑞特装</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -2869,17 +2869,17 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>002918</t>
+          <t>300349</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>蒙娜丽莎</t>
+          <t>金卡智能</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -2894,17 +2894,17 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>300349</t>
+          <t>002918</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>金卡智能</t>
+          <t>蒙娜丽莎</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">

</xml_diff>

<commit_message>
数据更新 2026-08-13（GitHub Actions 自动）
模式：daily

═══ 数据状态 ═══
  指数: 2026-08-13 ✓
  ETF: 2026-08-13 ✓
  推荐20: 2026-08-13 ✓
  其他成份: 2026-08-13 ✓
  自选: 2026-08-13 ✓
  成分样本: 2026-08-12 ⚠️ 滞后 1 天
  回测: 2026-08-10 ⚠️ 已过期（维护→1 重跑，约1分钟）
  季度检测: 从未执行（深度更新或维护可执行）
  失败清单: 2 只（北交所无数据源，预期内）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="980092" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="980092" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'980092'!$A$1:$E$101</definedName>

</xml_diff>

<commit_message>
数据更新 2026-08-18（GitHub Actions 自动）
模式：daily

═══ 数据状态 ═══
  指数: 2026-08-17 ✓
  ETF: 2026-08-17 ✓
  推荐20: 2026-08-17 ✓
  其他成份: 2026-08-17 ✓
  自选: 2026-08-17 ✓
  成分样本: 2026-08-17 ✓
  季度检测: 从未执行（深度更新或维护可执行）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9.58</v>
+        <v>9.550000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9.09</v>
+        <v>9.07</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6.3</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="5">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5.56</v>
+        <v>5.52</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.16</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="7">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>4.06</v>
+        <v>4.15</v>
       </c>
     </row>
     <row r="9">
@@ -650,17 +650,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>600050</t>
+          <t>000338</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>中国联通</t>
+          <t>潍柴动力</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>电信业务</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
@@ -673,21 +673,21 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>000338</t>
+          <t>600050</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>潍柴动力</t>
+          <t>中国联通</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>电信业务</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3.47</v>
+        <v>3.53</v>
       </c>
     </row>
     <row r="11">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3.28</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="12">
@@ -1269,17 +1269,17 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>600398</t>
+          <t>600352</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>海澜之家</t>
+          <t>浙江龙盛</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1294,17 +1294,17 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>600352</t>
+          <t>600398</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>浙江龙盛</t>
+          <t>海澜之家</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -1444,12 +1444,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>603883</t>
+          <t>600380</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>老百姓</t>
+          <t>健康元</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1469,12 +1469,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>600380</t>
+          <t>603883</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>健康元</t>
+          <t>老百姓</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1694,17 +1694,17 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>002761</t>
+          <t>603766</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>浙江建投</t>
+          <t>隆鑫通用</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -1719,17 +1719,17 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>603766</t>
+          <t>002761</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>隆鑫通用</t>
+          <t>浙江建投</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -1794,17 +1794,17 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>002039</t>
+          <t>002545</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>黔源电力</t>
+          <t>东方铁塔</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -1819,17 +1819,17 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>600729</t>
+          <t>002039</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>重百集团</t>
+          <t>黔源电力</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -1844,17 +1844,17 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>002545</t>
+          <t>600729</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>东方铁塔</t>
+          <t>重百集团</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -1894,17 +1894,17 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>002004</t>
+          <t>600004</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>华邦健康</t>
+          <t>白云机场</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -1919,17 +1919,17 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>600004</t>
+          <t>000957</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>白云机场</t>
+          <t>中通客车</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -1944,17 +1944,17 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>000957</t>
+          <t>002004</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>中通客车</t>
+          <t>华邦健康</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -2044,12 +2044,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>000090</t>
+          <t>002061</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>天健集团</t>
+          <t>浙江交科</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -2069,12 +2069,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>002061</t>
+          <t>000090</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>浙江交科</t>
+          <t>天健集团</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -2119,17 +2119,17 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>002563</t>
+          <t>002170</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>森马服饰</t>
+          <t>芭田股份</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -2144,17 +2144,17 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>002170</t>
+          <t>002563</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>芭田股份</t>
+          <t>森马服饰</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -2319,17 +2319,17 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>603708</t>
+          <t>002043</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>家家悦</t>
+          <t>兔 宝 宝</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -2344,17 +2344,17 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>002043</t>
+          <t>603708</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>兔 宝 宝</t>
+          <t>家家悦</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -2369,17 +2369,17 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>600686</t>
+          <t>600300</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>金龙汽车</t>
+          <t>维维股份</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -2394,17 +2394,17 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>600300</t>
+          <t>600686</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>维维股份</t>
+          <t>金龙汽车</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -2419,17 +2419,17 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>603368</t>
+          <t>603173</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>柳药集团</t>
+          <t>福斯达</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -2469,17 +2469,17 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>603173</t>
+          <t>603368</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>福斯达</t>
+          <t>柳药集团</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -2494,17 +2494,17 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>000650</t>
+          <t>605377</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>仁和药业</t>
+          <t>华旺科技</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -2519,17 +2519,17 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>605377</t>
+          <t>000650</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>华旺科技</t>
+          <t>仁和药业</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -2669,17 +2669,17 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>600897</t>
+          <t>600351</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>厦门空港</t>
+          <t>亚宝药业</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -2694,17 +2694,17 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>600351</t>
+          <t>600897</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>亚宝药业</t>
+          <t>厦门空港</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -2719,17 +2719,17 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>601002</t>
+          <t>000026</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>晋亿实业</t>
+          <t>飞亚达</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -2744,17 +2744,17 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>000026</t>
+          <t>002478</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>飞亚达</t>
+          <t>常宝股份</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -2769,17 +2769,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>300389</t>
+          <t>000551</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>艾比森</t>
+          <t>创元科技</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -2794,17 +2794,17 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>002478</t>
+          <t>002081</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>常宝股份</t>
+          <t>金 螳 螂</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -2819,12 +2819,12 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>300228</t>
+          <t>601002</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>富瑞特装</t>
+          <t>晋亿实业</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -2844,17 +2844,17 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>000551</t>
+          <t>300389</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>创元科技</t>
+          <t>艾比森</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -2869,12 +2869,12 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>002081</t>
+          <t>300228</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>金 螳 螂</t>
+          <t>富瑞特装</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">

</xml_diff>

<commit_message>
数据更新 2026-08-19（GitHub Actions 自动）
模式：daily

═══ 数据状态 ═══
  指数: 2026-08-18 ✓
  ETF: 2026-08-18 ✓
  推荐20: 2026-08-18 ✓
  其他成份: 2026-08-18 ✓
  自选: 2026-08-18 ✓
  成分样本: 2026-08-18 ✓
  季度检测: 从未执行（深度更新或维护可执行）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9.550000000000001</v>
+        <v>9.460000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9.07</v>
+        <v>9.220000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6.24</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="5">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5.52</v>
+        <v>5.46</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.1</v>
+        <v>5.05</v>
       </c>
     </row>
     <row r="7">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>4.31</v>
+        <v>4.33</v>
       </c>
     </row>
     <row r="8">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>4.15</v>
+        <v>4.09</v>
       </c>
     </row>
     <row r="9">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3.58</v>
+        <v>3.53</v>
       </c>
     </row>
     <row r="10">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3.53</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="11">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3.24</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="12">
@@ -1069,12 +1069,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>000959</t>
+          <t>600096</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>首钢股份</t>
+          <t>云天化</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1094,12 +1094,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>600096</t>
+          <t>000959</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>云天化</t>
+          <t>首钢股份</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1344,17 +1344,17 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>603444</t>
+          <t>600295</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>吉比特</t>
+          <t>鄂尔多斯</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -1369,17 +1369,17 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>600295</t>
+          <t>603444</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>鄂尔多斯</t>
+          <t>吉比特</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -1394,17 +1394,17 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>600320</t>
+          <t>600060</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>振华重工</t>
+          <t>海信视像</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -1419,17 +1419,17 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>600060</t>
+          <t>600320</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>海信视像</t>
+          <t>振华重工</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -1894,17 +1894,17 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>600004</t>
+          <t>000957</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>白云机场</t>
+          <t>中通客车</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -1919,17 +1919,17 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>000957</t>
+          <t>600004</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>中通客车</t>
+          <t>白云机场</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -1994,12 +1994,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>002416</t>
+          <t>000719</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>爱施德</t>
+          <t>中原传媒</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -2019,12 +2019,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>000719</t>
+          <t>002416</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>中原传媒</t>
+          <t>爱施德</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -2044,12 +2044,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>002061</t>
+          <t>000090</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>浙江交科</t>
+          <t>天健集团</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -2069,12 +2069,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>000090</t>
+          <t>002061</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>天健集团</t>
+          <t>浙江交科</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -2094,17 +2094,17 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>600163</t>
+          <t>002563</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>中闽能源</t>
+          <t>森马服饰</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -2144,17 +2144,17 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>002563</t>
+          <t>600163</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>森马服饰</t>
+          <t>中闽能源</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -2169,17 +2169,17 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>002204</t>
+          <t>000597</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>大连重工</t>
+          <t>东北制药</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -2194,17 +2194,17 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>000690</t>
+          <t>002204</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>宝新能源</t>
+          <t>大连重工</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -2219,17 +2219,17 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>000597</t>
+          <t>000690</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>东北制药</t>
+          <t>宝新能源</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -2269,17 +2269,17 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>000915</t>
+          <t>002697</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>华特达因</t>
+          <t>红旗连锁</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -2294,17 +2294,17 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>002697</t>
+          <t>000915</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>红旗连锁</t>
+          <t>华特达因</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
@@ -2319,17 +2319,17 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>002043</t>
+          <t>603708</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>兔 宝 宝</t>
+          <t>家家悦</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -2344,17 +2344,17 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>603708</t>
+          <t>002043</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>家家悦</t>
+          <t>兔 宝 宝</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -2394,17 +2394,17 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>600686</t>
+          <t>600195</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>金龙汽车</t>
+          <t>中牧股份</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -2444,17 +2444,17 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>600195</t>
+          <t>600686</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>中牧股份</t>
+          <t>金龙汽车</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -2494,17 +2494,17 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>605377</t>
+          <t>000650</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>华旺科技</t>
+          <t>仁和药业</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -2519,17 +2519,17 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>000650</t>
+          <t>601801</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>仁和药业</t>
+          <t>皖新传媒</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -2544,17 +2544,17 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>601801</t>
+          <t>605377</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>皖新传媒</t>
+          <t>华旺科技</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -2594,17 +2594,17 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>002390</t>
+          <t>001338</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>信邦制药</t>
+          <t>永顺泰</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
@@ -2619,17 +2619,17 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>001338</t>
+          <t>002390</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>永顺泰</t>
+          <t>信邦制药</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -2744,17 +2744,17 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>002478</t>
+          <t>002081</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>常宝股份</t>
+          <t>金 螳 螂</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -2769,17 +2769,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>000551</t>
+          <t>002478</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>创元科技</t>
+          <t>常宝股份</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -2794,12 +2794,12 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>002081</t>
+          <t>601002</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>金 螳 螂</t>
+          <t>晋亿实业</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -2819,17 +2819,17 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>601002</t>
+          <t>300389</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>晋亿实业</t>
+          <t>艾比森</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -2844,17 +2844,17 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>300389</t>
+          <t>300228</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>艾比森</t>
+          <t>富瑞特装</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -2869,12 +2869,12 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>300228</t>
+          <t>000551</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>富瑞特装</t>
+          <t>创元科技</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">

</xml_diff>

<commit_message>
数据更新 2026-08-20（GitHub Actions 自动）
模式：daily

═══ 数据状态 ═══
  指数: 2026-08-20 ✓
  ETF: 2026-08-19 ⚠️ 滞后 1 天
  推荐20: 2026-08-20 ✓
  其他成份: 2026-08-19 ⚠️ 滞后 1 天
  自选: 2026-08-20 ✓
  成分样本: 2026-08-19 ⚠️ 滞后 1 天
  季度检测: 从未执行（深度更新或维护可执行）
  失败清单: 52 只（52 只可重试，维护→2 重试）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9.460000000000001</v>
+        <v>9.66</v>
       </c>
     </row>
     <row r="3">
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9.220000000000001</v>
+        <v>9.24</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6.25</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="5">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5.46</v>
+        <v>5.47</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.05</v>
+        <v>5.08</v>
       </c>
     </row>
     <row r="7">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>4.33</v>
+        <v>4.21</v>
       </c>
     </row>
     <row r="8">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>4.09</v>
+        <v>4.08</v>
       </c>
     </row>
     <row r="9">
@@ -650,21 +650,21 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>000338</t>
+          <t>600050</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>潍柴动力</t>
+          <t>中国联通</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>电信业务</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3.53</v>
+        <v>3.42</v>
       </c>
     </row>
     <row r="10">
@@ -673,21 +673,21 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>600050</t>
+          <t>000338</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>中国联通</t>
+          <t>潍柴动力</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>电信业务</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3.5</v>
+        <v>3.31</v>
       </c>
     </row>
     <row r="11">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3.21</v>
+        <v>3.12</v>
       </c>
     </row>
     <row r="12">
@@ -1269,17 +1269,17 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>600352</t>
+          <t>600398</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>浙江龙盛</t>
+          <t>海澜之家</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1294,17 +1294,17 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>600398</t>
+          <t>600352</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>海澜之家</t>
+          <t>浙江龙盛</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -1319,17 +1319,17 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>688819</t>
+          <t>600295</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>天能股份</t>
+          <t>鄂尔多斯</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1344,17 +1344,17 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>600295</t>
+          <t>688819</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>鄂尔多斯</t>
+          <t>天能股份</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -1619,17 +1619,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>601001</t>
+          <t>601083</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>晋控煤业</t>
+          <t>锦江航运</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -1644,17 +1644,17 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>601083</t>
+          <t>601001</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>锦江航运</t>
+          <t>晋控煤业</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -1669,17 +1669,17 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>300244</t>
+          <t>603766</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>迪安诊断</t>
+          <t>隆鑫通用</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -1694,17 +1694,17 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>603766</t>
+          <t>002761</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>隆鑫通用</t>
+          <t>浙江建投</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -1719,17 +1719,17 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>002761</t>
+          <t>300244</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>浙江建投</t>
+          <t>迪安诊断</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -1894,17 +1894,17 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>000957</t>
+          <t>600004</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>中通客车</t>
+          <t>白云机场</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -1919,17 +1919,17 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>600004</t>
+          <t>002004</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>白云机场</t>
+          <t>华邦健康</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -1944,17 +1944,17 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>002004</t>
+          <t>000957</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>华邦健康</t>
+          <t>中通客车</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -1969,17 +1969,17 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>002727</t>
+          <t>000719</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>一心堂</t>
+          <t>中原传媒</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -1994,17 +1994,17 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>000719</t>
+          <t>002727</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>中原传媒</t>
+          <t>一心堂</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -2019,17 +2019,17 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>002416</t>
+          <t>002061</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>爱施德</t>
+          <t>浙江交科</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -2069,17 +2069,17 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>002061</t>
+          <t>002416</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>浙江交科</t>
+          <t>爱施德</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -2119,17 +2119,17 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>002170</t>
+          <t>600163</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>芭田股份</t>
+          <t>中闽能源</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -2144,17 +2144,17 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>600163</t>
+          <t>002170</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>中闽能源</t>
+          <t>芭田股份</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -2169,17 +2169,17 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>000597</t>
+          <t>000690</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>东北制药</t>
+          <t>宝新能源</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -2219,17 +2219,17 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>000690</t>
+          <t>000597</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>宝新能源</t>
+          <t>东北制药</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -2269,17 +2269,17 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>002697</t>
+          <t>000915</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>红旗连锁</t>
+          <t>华特达因</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -2294,17 +2294,17 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>000915</t>
+          <t>002697</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>华特达因</t>
+          <t>红旗连锁</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
@@ -2319,17 +2319,17 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>603708</t>
+          <t>002043</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>家家悦</t>
+          <t>兔 宝 宝</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -2344,17 +2344,17 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>002043</t>
+          <t>603708</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>兔 宝 宝</t>
+          <t>家家悦</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -2419,17 +2419,17 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>603173</t>
+          <t>603368</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>福斯达</t>
+          <t>柳药集团</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -2444,17 +2444,17 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>600686</t>
+          <t>603173</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>金龙汽车</t>
+          <t>福斯达</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -2469,17 +2469,17 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>603368</t>
+          <t>600686</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>柳药集团</t>
+          <t>金龙汽车</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -2494,17 +2494,17 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>000650</t>
+          <t>601801</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>仁和药业</t>
+          <t>皖新传媒</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -2519,17 +2519,17 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>601801</t>
+          <t>000650</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>皖新传媒</t>
+          <t>仁和药业</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -2569,17 +2569,17 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>603279</t>
+          <t>001338</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>景津装备</t>
+          <t>永顺泰</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -2594,17 +2594,17 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>001338</t>
+          <t>603279</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>永顺泰</t>
+          <t>景津装备</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
@@ -2669,17 +2669,17 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>600351</t>
+          <t>600897</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>亚宝药业</t>
+          <t>厦门空港</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -2694,17 +2694,17 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>600897</t>
+          <t>600351</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>厦门空港</t>
+          <t>亚宝药业</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -2744,17 +2744,17 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>002081</t>
+          <t>002478</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>金 螳 螂</t>
+          <t>常宝股份</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -2769,17 +2769,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>002478</t>
+          <t>002081</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>常宝股份</t>
+          <t>金 螳 螂</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -2869,12 +2869,12 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>000551</t>
+          <t>002918</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>创元科技</t>
+          <t>蒙娜丽莎</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -2894,17 +2894,17 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>002918</t>
+          <t>300349</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>蒙娜丽莎</t>
+          <t>金卡智能</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
@@ -2919,17 +2919,17 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>300349</t>
+          <t>000551</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>金卡智能</t>
+          <t>创元科技</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">

</xml_diff>

<commit_message>
数据更新 2026-08-21（GitHub Actions 自动）
模式：daily

═══ 数据状态 ═══
  指数: 2026-08-21 ✓
  ETF: 2026-08-21 ✓
  推荐20: 2026-08-21 ✓
  其他成份: 2026-08-21 ✓
  自选: 2026-08-21 ✓
  成分样本: 2026-08-20 ⚠️ 滞后 1 天
  季度检测: 从未执行（深度更新或维护可执行）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9.66</v>
+        <v>9.49</v>
       </c>
     </row>
     <row r="3">
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9.24</v>
+        <v>9.19</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6.5</v>
+        <v>6.49</v>
       </c>
     </row>
     <row r="5">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5.47</v>
+        <v>5.53</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.08</v>
+        <v>5.16</v>
       </c>
     </row>
     <row r="7">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>4.21</v>
+        <v>4.18</v>
       </c>
     </row>
     <row r="8">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>4.08</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="9">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3.42</v>
+        <v>3.47</v>
       </c>
     </row>
     <row r="10">
@@ -673,12 +673,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>000338</t>
+          <t>601877</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>潍柴动力</t>
+          <t>正泰电器</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3.31</v>
+        <v>3.42</v>
       </c>
     </row>
     <row r="11">
@@ -696,12 +696,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>601877</t>
+          <t>000338</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>正泰电器</t>
+          <t>潍柴动力</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3.12</v>
+        <v>3.29</v>
       </c>
     </row>
     <row r="12">
@@ -1069,12 +1069,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>600096</t>
+          <t>000959</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>云天化</t>
+          <t>首钢股份</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1094,12 +1094,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>000959</t>
+          <t>600096</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>首钢股份</t>
+          <t>云天化</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1669,17 +1669,17 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>603766</t>
+          <t>300244</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>隆鑫通用</t>
+          <t>迪安诊断</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -1694,17 +1694,17 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>002761</t>
+          <t>603766</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>浙江建投</t>
+          <t>隆鑫通用</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -1719,17 +1719,17 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>300244</t>
+          <t>002761</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>迪安诊断</t>
+          <t>浙江建投</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -1794,17 +1794,17 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>002545</t>
+          <t>600729</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>东方铁塔</t>
+          <t>重百集团</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>600729</t>
+          <t>601339</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>重百集团</t>
+          <t>百隆东方</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -1869,17 +1869,17 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>601339</t>
+          <t>002545</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>百隆东方</t>
+          <t>东方铁塔</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -1969,17 +1969,17 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>000719</t>
+          <t>002727</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>中原传媒</t>
+          <t>一心堂</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -1994,17 +1994,17 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>002727</t>
+          <t>000719</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>一心堂</t>
+          <t>中原传媒</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -2019,12 +2019,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>002061</t>
+          <t>000090</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>浙江交科</t>
+          <t>天健集团</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -2044,12 +2044,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>000090</t>
+          <t>002061</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>天健集团</t>
+          <t>浙江交科</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -2294,17 +2294,17 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>002697</t>
+          <t>002043</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>红旗连锁</t>
+          <t>兔 宝 宝</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
@@ -2319,17 +2319,17 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>002043</t>
+          <t>002697</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>兔 宝 宝</t>
+          <t>红旗连锁</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -2369,12 +2369,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>600300</t>
+          <t>600195</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>维维股份</t>
+          <t>中牧股份</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -2394,12 +2394,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>600195</t>
+          <t>600300</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>中牧股份</t>
+          <t>维维股份</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -2494,17 +2494,17 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>601801</t>
+          <t>000650</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>皖新传媒</t>
+          <t>仁和药业</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -2519,17 +2519,17 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>000650</t>
+          <t>601801</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>仁和药业</t>
+          <t>皖新传媒</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -2569,17 +2569,17 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>001338</t>
+          <t>603279</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>永顺泰</t>
+          <t>景津装备</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -2594,17 +2594,17 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>603279</t>
+          <t>001338</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>景津装备</t>
+          <t>永顺泰</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
@@ -2669,17 +2669,17 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>600897</t>
+          <t>600351</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>厦门空港</t>
+          <t>亚宝药业</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -2694,17 +2694,17 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>600351</t>
+          <t>600897</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>亚宝药业</t>
+          <t>厦门空港</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -2744,17 +2744,17 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>002478</t>
+          <t>601002</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>常宝股份</t>
+          <t>晋亿实业</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -2769,17 +2769,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>002081</t>
+          <t>002478</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>金 螳 螂</t>
+          <t>常宝股份</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -2794,12 +2794,12 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>601002</t>
+          <t>002081</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>晋亿实业</t>
+          <t>金 螳 螂</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">

</xml_diff>

<commit_message>
数据更新 2026-08-24（GitHub Actions 自动）
模式：weekly

═══ 数据状态 ═══
  指数: 2026-08-24 ✓
  ETF: 2026-08-24 ✓
  推荐20: 2026-08-24 ✓
  其他成份: 2026-08-24 ✓
  自选: 2026-08-24 ✓
  成分样本: 2026-08-21 ⚠️ 滞后 3 天
  季度检测: 从未执行（深度更新或维护可执行）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -489,21 +489,21 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>601728</t>
+          <t>600938</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>中国电信</t>
+          <t>中国海油</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>电信业务</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9.49</v>
+        <v>9.359999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -512,21 +512,21 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>600938</t>
+          <t>601728</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>中国海油</t>
+          <t>中国电信</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>电信业务</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9.19</v>
+        <v>9.32</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6.49</v>
+        <v>6.47</v>
       </c>
     </row>
     <row r="5">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5.53</v>
+        <v>5.42</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.16</v>
+        <v>5.15</v>
       </c>
     </row>
     <row r="7">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>4.18</v>
+        <v>4.19</v>
       </c>
     </row>
     <row r="8">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>3.99</v>
+        <v>4.11</v>
       </c>
     </row>
     <row r="9">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3.47</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="10">
@@ -673,12 +673,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>601877</t>
+          <t>000338</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>正泰电器</t>
+          <t>潍柴动力</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3.42</v>
+        <v>3.39</v>
       </c>
     </row>
     <row r="11">
@@ -696,12 +696,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>000338</t>
+          <t>601877</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>潍柴动力</t>
+          <t>正泰电器</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3.29</v>
+        <v>3.37</v>
       </c>
     </row>
     <row r="12">
@@ -1219,17 +1219,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>000921</t>
+          <t>600546</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>海信家电</t>
+          <t>山煤国际</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1244,17 +1244,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>600546</t>
+          <t>000921</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>山煤国际</t>
+          <t>海信家电</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1319,17 +1319,17 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>600295</t>
+          <t>688819</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>鄂尔多斯</t>
+          <t>天能股份</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1344,17 +1344,17 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>688819</t>
+          <t>600295</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>天能股份</t>
+          <t>鄂尔多斯</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -1444,17 +1444,17 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>600380</t>
+          <t>603565</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>健康元</t>
+          <t>中谷物流</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -1494,17 +1494,17 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>603565</t>
+          <t>600380</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>中谷物流</t>
+          <t>健康元</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -1544,17 +1544,17 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>000513</t>
+          <t>600874</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>丽珠集团</t>
+          <t>创业环保</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -1569,17 +1569,17 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>600874</t>
+          <t>000513</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>创业环保</t>
+          <t>丽珠集团</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -1594,17 +1594,17 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>600267</t>
+          <t>601083</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>海正药业</t>
+          <t>锦江航运</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -1619,17 +1619,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>601083</t>
+          <t>600267</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>锦江航运</t>
+          <t>海正药业</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -1794,17 +1794,17 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>600729</t>
+          <t>002039</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>重百集团</t>
+          <t>黔源电力</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -1819,17 +1819,17 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>002039</t>
+          <t>002545</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>黔源电力</t>
+          <t>东方铁塔</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -1869,17 +1869,17 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>002545</t>
+          <t>600729</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>东方铁塔</t>
+          <t>重百集团</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -2044,17 +2044,17 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>002061</t>
+          <t>002416</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>浙江交科</t>
+          <t>爱施德</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -2069,17 +2069,17 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>002416</t>
+          <t>002061</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>爱施德</t>
+          <t>浙江交科</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -2094,17 +2094,17 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>002563</t>
+          <t>002170</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>森马服饰</t>
+          <t>芭田股份</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -2144,17 +2144,17 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>002170</t>
+          <t>002563</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>芭田股份</t>
+          <t>森马服饰</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -2269,17 +2269,17 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>000915</t>
+          <t>002697</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>华特达因</t>
+          <t>红旗连锁</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -2319,17 +2319,17 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>002697</t>
+          <t>000915</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>红旗连锁</t>
+          <t>华特达因</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -2419,17 +2419,17 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>603368</t>
+          <t>603173</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>柳药集团</t>
+          <t>福斯达</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -2444,17 +2444,17 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>603173</t>
+          <t>600686</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>福斯达</t>
+          <t>金龙汽车</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -2469,17 +2469,17 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>600686</t>
+          <t>603368</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>金龙汽车</t>
+          <t>柳药集团</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -2494,17 +2494,17 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>000650</t>
+          <t>601801</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>仁和药业</t>
+          <t>皖新传媒</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -2519,17 +2519,17 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>601801</t>
+          <t>000650</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>皖新传媒</t>
+          <t>仁和药业</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -2669,17 +2669,17 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>600351</t>
+          <t>600897</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>亚宝药业</t>
+          <t>厦门空港</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -2694,17 +2694,17 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>600897</t>
+          <t>600351</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>厦门空港</t>
+          <t>亚宝药业</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -2794,17 +2794,17 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>002081</t>
+          <t>300389</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>金 螳 螂</t>
+          <t>艾比森</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -2819,17 +2819,17 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>300389</t>
+          <t>300228</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>艾比森</t>
+          <t>富瑞特装</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -2844,12 +2844,12 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>300228</t>
+          <t>002918</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>富瑞特装</t>
+          <t>蒙娜丽莎</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -2869,12 +2869,12 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>002918</t>
+          <t>002081</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>蒙娜丽莎</t>
+          <t>金 螳 螂</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">

</xml_diff>

<commit_message>
数据更新 2026-08-25（GitHub Actions 自动）
模式：daily

═══ 数据状态 ═══
  指数: 2026-08-25 ✓
  ETF: 2026-08-25 ✓
  推荐20: 2026-08-25 ✓
  其他成份: 2026-08-25 ✓
  自选: 2026-08-25 ✓
  成分样本: 2026-08-24 ⚠️ 滞后 1 天
  季度检测: 从未执行（深度更新或维护可执行）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -489,21 +489,21 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>600938</t>
+          <t>601728</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>中国海油</t>
+          <t>中国电信</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>电信业务</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9.359999999999999</v>
+        <v>9.369999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -512,17 +512,17 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>601728</t>
+          <t>600938</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>中国电信</t>
+          <t>中国海油</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>电信业务</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6.47</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="5">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.15</v>
+        <v>5.17</v>
       </c>
     </row>
     <row r="7">
@@ -604,21 +604,21 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>000100</t>
+          <t>601600</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>TCL科技</t>
+          <t>中国铝业</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>4.19</v>
+        <v>4.14</v>
       </c>
     </row>
     <row r="8">
@@ -627,21 +627,21 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>601600</t>
+          <t>000100</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>中国铝业</t>
+          <t>TCL科技</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>4.11</v>
+        <v>4.09</v>
       </c>
     </row>
     <row r="9">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3.45</v>
+        <v>3.48</v>
       </c>
     </row>
     <row r="10">
@@ -673,12 +673,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>000338</t>
+          <t>601877</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>潍柴动力</t>
+          <t>正泰电器</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3.39</v>
+        <v>3.42</v>
       </c>
     </row>
     <row r="11">
@@ -696,12 +696,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>601877</t>
+          <t>000338</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>正泰电器</t>
+          <t>潍柴动力</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3.37</v>
+        <v>3.14</v>
       </c>
     </row>
     <row r="12">
@@ -1194,17 +1194,17 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>601880</t>
+          <t>600546</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>辽港股份</t>
+          <t>山煤国际</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1219,17 +1219,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>600546</t>
+          <t>601880</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>山煤国际</t>
+          <t>辽港股份</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1244,12 +1244,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>000921</t>
+          <t>600398</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>海信家电</t>
+          <t>海澜之家</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1269,12 +1269,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>600398</t>
+          <t>000921</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>海澜之家</t>
+          <t>海信家电</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1394,17 +1394,17 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>600060</t>
+          <t>603565</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>海信视像</t>
+          <t>中谷物流</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -1444,17 +1444,17 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>603565</t>
+          <t>600060</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>中谷物流</t>
+          <t>海信视像</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -1544,17 +1544,17 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>600874</t>
+          <t>601083</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>创业环保</t>
+          <t>锦江航运</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -1569,17 +1569,17 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>000513</t>
+          <t>600874</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>丽珠集团</t>
+          <t>创业环保</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -1594,17 +1594,17 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>601083</t>
+          <t>000513</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>锦江航运</t>
+          <t>丽珠集团</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -1619,17 +1619,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>600267</t>
+          <t>603766</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>海正药业</t>
+          <t>隆鑫通用</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -1694,17 +1694,17 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>603766</t>
+          <t>600267</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>隆鑫通用</t>
+          <t>海正药业</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>601339</t>
+          <t>600729</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>百隆东方</t>
+          <t>重百集团</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -1869,12 +1869,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>600729</t>
+          <t>601339</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>重百集团</t>
+          <t>百隆东方</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -1919,17 +1919,17 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>002004</t>
+          <t>000957</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>华邦健康</t>
+          <t>中通客车</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -1944,17 +1944,17 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>000957</t>
+          <t>002004</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>中通客车</t>
+          <t>华邦健康</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -2019,12 +2019,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>000090</t>
+          <t>002061</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>天健集团</t>
+          <t>浙江交科</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -2069,12 +2069,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>002061</t>
+          <t>000090</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>浙江交科</t>
+          <t>天健集团</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -2094,17 +2094,17 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>002170</t>
+          <t>002563</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>芭田股份</t>
+          <t>森马服饰</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -2144,17 +2144,17 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>002563</t>
+          <t>002170</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>森马服饰</t>
+          <t>芭田股份</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -2219,17 +2219,17 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>000597</t>
+          <t>301039</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>东北制药</t>
+          <t>中集车辆</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -2244,17 +2244,17 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>301039</t>
+          <t>000597</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>中集车辆</t>
+          <t>东北制药</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -2269,17 +2269,17 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>002697</t>
+          <t>002043</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>红旗连锁</t>
+          <t>兔 宝 宝</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -2294,17 +2294,17 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>002043</t>
+          <t>002697</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>兔 宝 宝</t>
+          <t>红旗连锁</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
@@ -2494,17 +2494,17 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>601801</t>
+          <t>605377</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>皖新传媒</t>
+          <t>华旺科技</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -2519,17 +2519,17 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>000650</t>
+          <t>601801</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>仁和药业</t>
+          <t>皖新传媒</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -2544,17 +2544,17 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>605377</t>
+          <t>000650</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>华旺科技</t>
+          <t>仁和药业</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -2719,17 +2719,17 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>000026</t>
+          <t>601002</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>飞亚达</t>
+          <t>晋亿实业</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -2744,17 +2744,17 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>601002</t>
+          <t>002478</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>晋亿实业</t>
+          <t>常宝股份</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -2769,17 +2769,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>002478</t>
+          <t>300389</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>常宝股份</t>
+          <t>艾比森</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -2794,17 +2794,17 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>300389</t>
+          <t>000026</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>艾比森</t>
+          <t>飞亚达</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">

</xml_diff>

<commit_message>
数据更新 2026-08-26（GitHub Actions 自动）
模式：daily

═══ 数据状态 ═══
  指数: 2026-08-26 ✓
  ETF: 2026-08-26 ✓
  推荐20: 2026-08-26 ✓
  其他成份: 2026-08-26 ✓
  自选: 2026-08-26 ✓
  成分样本: 2026-08-25 ⚠️ 滞后 1 天
  季度检测: 从未执行（深度更新或维护可执行）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9.369999999999999</v>
+        <v>9.33</v>
       </c>
     </row>
     <row r="3">
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9.32</v>
+        <v>9.24</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6.5</v>
+        <v>6.52</v>
       </c>
     </row>
     <row r="5">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5.42</v>
+        <v>5.47</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.17</v>
+        <v>5.22</v>
       </c>
     </row>
     <row r="7">
@@ -604,21 +604,21 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>601600</t>
+          <t>000100</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>中国铝业</t>
+          <t>TCL科技</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>4.14</v>
+        <v>4.08</v>
       </c>
     </row>
     <row r="8">
@@ -627,21 +627,21 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>000100</t>
+          <t>601600</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>TCL科技</t>
+          <t>中国铝业</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>4.09</v>
+        <v>4.07</v>
       </c>
     </row>
     <row r="9">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3.48</v>
+        <v>3.54</v>
       </c>
     </row>
     <row r="10">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3.42</v>
+        <v>3.38</v>
       </c>
     </row>
     <row r="11">
@@ -1194,17 +1194,17 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>600546</t>
+          <t>601880</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>山煤国际</t>
+          <t>辽港股份</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1219,17 +1219,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>601880</t>
+          <t>000921</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>辽港股份</t>
+          <t>海信家电</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1244,17 +1244,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>600398</t>
+          <t>600546</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>海澜之家</t>
+          <t>山煤国际</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1269,12 +1269,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>000921</t>
+          <t>600398</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>海信家电</t>
+          <t>海澜之家</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1394,17 +1394,17 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>603565</t>
+          <t>600060</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>中谷物流</t>
+          <t>海信视像</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -1444,17 +1444,17 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>600060</t>
+          <t>603565</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>海信视像</t>
+          <t>中谷物流</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -1594,17 +1594,17 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>000513</t>
+          <t>603766</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>丽珠集团</t>
+          <t>隆鑫通用</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -1619,17 +1619,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>603766</t>
+          <t>601001</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>隆鑫通用</t>
+          <t>晋控煤业</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -1644,17 +1644,17 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>601001</t>
+          <t>000513</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>晋控煤业</t>
+          <t>丽珠集团</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -1669,12 +1669,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>300244</t>
+          <t>600267</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>迪安诊断</t>
+          <t>海正药业</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -1694,17 +1694,17 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>600267</t>
+          <t>002761</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>海正药业</t>
+          <t>浙江建投</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -1719,17 +1719,17 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>002761</t>
+          <t>300244</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>浙江建投</t>
+          <t>迪安诊断</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -1819,17 +1819,17 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>002545</t>
+          <t>600729</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>东方铁塔</t>
+          <t>重百集团</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>600729</t>
+          <t>601339</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>重百集团</t>
+          <t>百隆东方</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -1869,17 +1869,17 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>601339</t>
+          <t>002545</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>百隆东方</t>
+          <t>东方铁塔</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -1919,17 +1919,17 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>000957</t>
+          <t>002004</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>中通客车</t>
+          <t>华邦健康</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -1944,17 +1944,17 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>002004</t>
+          <t>000957</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>华邦健康</t>
+          <t>中通客车</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -2044,17 +2044,17 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>002416</t>
+          <t>000090</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>爱施德</t>
+          <t>天健集团</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -2069,17 +2069,17 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>000090</t>
+          <t>002416</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>天健集团</t>
+          <t>爱施德</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -2269,17 +2269,17 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>002043</t>
+          <t>002697</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>兔 宝 宝</t>
+          <t>红旗连锁</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -2294,17 +2294,17 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>002697</t>
+          <t>000915</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>红旗连锁</t>
+          <t>华特达因</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
@@ -2319,17 +2319,17 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>000915</t>
+          <t>002043</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>华特达因</t>
+          <t>兔 宝 宝</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -2419,17 +2419,17 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>603173</t>
+          <t>600686</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>福斯达</t>
+          <t>金龙汽车</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -2444,17 +2444,17 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>600686</t>
+          <t>603173</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>金龙汽车</t>
+          <t>福斯达</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -2494,17 +2494,17 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>605377</t>
+          <t>000650</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>华旺科技</t>
+          <t>仁和药业</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -2544,17 +2544,17 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>000650</t>
+          <t>605377</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>仁和药业</t>
+          <t>华旺科技</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -2669,17 +2669,17 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>600897</t>
+          <t>600351</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>厦门空港</t>
+          <t>亚宝药业</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -2694,17 +2694,17 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>600351</t>
+          <t>600897</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>亚宝药业</t>
+          <t>厦门空港</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -2719,17 +2719,17 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>601002</t>
+          <t>002478</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>晋亿实业</t>
+          <t>常宝股份</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -2744,17 +2744,17 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>002478</t>
+          <t>601002</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>常宝股份</t>
+          <t>晋亿实业</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -2794,17 +2794,17 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>000026</t>
+          <t>002081</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>飞亚达</t>
+          <t>金 螳 螂</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -2819,17 +2819,17 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>300228</t>
+          <t>000026</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>富瑞特装</t>
+          <t>飞亚达</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -2844,12 +2844,12 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>002918</t>
+          <t>300228</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>蒙娜丽莎</t>
+          <t>富瑞特装</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -2869,12 +2869,12 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>002081</t>
+          <t>002918</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>金 螳 螂</t>
+          <t>蒙娜丽莎</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">

</xml_diff>

<commit_message>
数据更新 2026-08-27（GitHub Actions 自动）
模式：daily

═══ 数据状态 ═══
  指数: 2026-08-27 ✓
  ETF: 2026-08-27 ✓
  推荐20: 2026-08-27 ✓
  其他成份: 2026-08-27 ✓
  自选: 2026-08-27 ✓
  成分样本: 2026-08-26 ⚠️ 滞后 1 天
  季度检测: 从未执行（深度更新或维护可执行）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9.33</v>
+        <v>9.25</v>
       </c>
     </row>
     <row r="3">
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9.24</v>
+        <v>9.16</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6.52</v>
+        <v>6.49</v>
       </c>
     </row>
     <row r="5">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5.47</v>
+        <v>5.46</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.22</v>
+        <v>5.25</v>
       </c>
     </row>
     <row r="7">
@@ -604,21 +604,21 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>000100</t>
+          <t>601600</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>TCL科技</t>
+          <t>中国铝业</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>4.08</v>
+        <v>4.16</v>
       </c>
     </row>
     <row r="8">
@@ -627,17 +627,17 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>601600</t>
+          <t>000100</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>中国铝业</t>
+          <t>TCL科技</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3.54</v>
+        <v>3.51</v>
       </c>
     </row>
     <row r="10">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3.38</v>
+        <v>3.37</v>
       </c>
     </row>
     <row r="11">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3.14</v>
+        <v>3.13</v>
       </c>
     </row>
     <row r="12">
@@ -1219,17 +1219,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>000921</t>
+          <t>600546</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>海信家电</t>
+          <t>山煤国际</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1244,17 +1244,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>600546</t>
+          <t>000921</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>山煤国际</t>
+          <t>海信家电</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1294,12 +1294,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>600352</t>
+          <t>600295</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>浙江龙盛</t>
+          <t>鄂尔多斯</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1344,12 +1344,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>600295</t>
+          <t>600352</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>鄂尔多斯</t>
+          <t>浙江龙盛</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1369,17 +1369,17 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>603444</t>
+          <t>600060</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>吉比特</t>
+          <t>海信视像</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -1394,17 +1394,17 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>600060</t>
+          <t>603444</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>海信视像</t>
+          <t>吉比特</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -1544,17 +1544,17 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>601083</t>
+          <t>600874</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>锦江航运</t>
+          <t>创业环保</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -1569,17 +1569,17 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>600874</t>
+          <t>601083</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>创业环保</t>
+          <t>锦江航运</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -1594,17 +1594,17 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>603766</t>
+          <t>601001</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>隆鑫通用</t>
+          <t>晋控煤业</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -1619,17 +1619,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>601001</t>
+          <t>603766</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>晋控煤业</t>
+          <t>隆鑫通用</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -1719,17 +1719,17 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>300244</t>
+          <t>600033</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>迪安诊断</t>
+          <t>福建高速</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -1744,12 +1744,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>600033</t>
+          <t>000400</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>福建高速</t>
+          <t>许继电气</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -1769,17 +1769,17 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>000400</t>
+          <t>300244</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>许继电气</t>
+          <t>迪安诊断</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -1844,17 +1844,17 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>601339</t>
+          <t>002545</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>百隆东方</t>
+          <t>东方铁塔</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -1869,17 +1869,17 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>002545</t>
+          <t>600004</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>东方铁塔</t>
+          <t>白云机场</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -1894,17 +1894,17 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>600004</t>
+          <t>601339</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>白云机场</t>
+          <t>百隆东方</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -1994,17 +1994,17 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>000719</t>
+          <t>002061</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>中原传媒</t>
+          <t>浙江交科</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -2019,17 +2019,17 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>002061</t>
+          <t>000719</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>浙江交科</t>
+          <t>中原传媒</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -2094,17 +2094,17 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>002563</t>
+          <t>600163</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>森马服饰</t>
+          <t>中闽能源</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -2119,17 +2119,17 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>600163</t>
+          <t>002563</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>中闽能源</t>
+          <t>森马服饰</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">

</xml_diff>

<commit_message>
数据更新 2026-08-28（GitHub Actions 自动）
模式：daily

═══ 数据状态 ═══
  指数: 2026-08-27 ✓
  ETF: 2026-08-27 ✓
  推荐20: 2026-08-27 ✓
  其他成份: 2026-08-27 ✓
  自选: 2026-08-27 ✓
  成分样本: 2026-08-27 ✓
  季度检测: 从未执行（深度更新或维护可执行）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -489,21 +489,21 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>601728</t>
+          <t>600938</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>中国电信</t>
+          <t>中国海油</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>电信业务</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9.25</v>
+        <v>9.32</v>
       </c>
     </row>
     <row r="3">
@@ -512,21 +512,21 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>600938</t>
+          <t>601728</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>中国海油</t>
+          <t>中国电信</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>电信业务</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9.16</v>
+        <v>9.18</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6.49</v>
+        <v>6.14</v>
       </c>
     </row>
     <row r="5">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5.46</v>
+        <v>5.43</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.25</v>
+        <v>5.18</v>
       </c>
     </row>
     <row r="7">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>4.16</v>
+        <v>4.19</v>
       </c>
     </row>
     <row r="8">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>4.07</v>
+        <v>4.13</v>
       </c>
     </row>
     <row r="9">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3.51</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="10">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3.37</v>
+        <v>3.35</v>
       </c>
     </row>
     <row r="11">
@@ -1069,12 +1069,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>000959</t>
+          <t>600096</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>首钢股份</t>
+          <t>云天化</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1094,12 +1094,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>600096</t>
+          <t>000959</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>云天化</t>
+          <t>首钢股份</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1194,17 +1194,17 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>601880</t>
+          <t>600546</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>辽港股份</t>
+          <t>山煤国际</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1219,17 +1219,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>600546</t>
+          <t>601880</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>山煤国际</t>
+          <t>辽港股份</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1319,17 +1319,17 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>688819</t>
+          <t>600352</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>天能股份</t>
+          <t>浙江龙盛</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1344,17 +1344,17 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>600352</t>
+          <t>688819</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>浙江龙盛</t>
+          <t>天能股份</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -1544,17 +1544,17 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>600874</t>
+          <t>601083</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>创业环保</t>
+          <t>锦江航运</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -1569,17 +1569,17 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>601083</t>
+          <t>600874</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>锦江航运</t>
+          <t>创业环保</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -1619,17 +1619,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>603766</t>
+          <t>000513</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>隆鑫通用</t>
+          <t>丽珠集团</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -1644,17 +1644,17 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>000513</t>
+          <t>603766</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>丽珠集团</t>
+          <t>隆鑫通用</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -1794,17 +1794,17 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>002039</t>
+          <t>002545</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>黔源电力</t>
+          <t>东方铁塔</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -1819,17 +1819,17 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>600729</t>
+          <t>002039</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>重百集团</t>
+          <t>黔源电力</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -1844,17 +1844,17 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>002545</t>
+          <t>600729</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>东方铁塔</t>
+          <t>重百集团</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -1894,17 +1894,17 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>601339</t>
+          <t>002004</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>百隆东方</t>
+          <t>华邦健康</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -1919,17 +1919,17 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>002004</t>
+          <t>601339</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>华邦健康</t>
+          <t>百隆东方</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -1969,17 +1969,17 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>002727</t>
+          <t>002061</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>一心堂</t>
+          <t>浙江交科</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -1994,12 +1994,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>002061</t>
+          <t>000090</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>浙江交科</t>
+          <t>天健集团</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -2019,17 +2019,17 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>000719</t>
+          <t>002727</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>中原传媒</t>
+          <t>一心堂</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -2044,17 +2044,17 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>000090</t>
+          <t>002416</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>天健集团</t>
+          <t>爱施德</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -2069,12 +2069,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>002416</t>
+          <t>000719</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>爱施德</t>
+          <t>中原传媒</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -2094,17 +2094,17 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>600163</t>
+          <t>002170</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>中闽能源</t>
+          <t>芭田股份</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -2119,17 +2119,17 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>002563</t>
+          <t>600163</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>森马服饰</t>
+          <t>中闽能源</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -2144,17 +2144,17 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>002170</t>
+          <t>002563</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>芭田股份</t>
+          <t>森马服饰</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -2219,17 +2219,17 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>301039</t>
+          <t>000597</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>中集车辆</t>
+          <t>东北制药</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -2244,17 +2244,17 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>000597</t>
+          <t>301039</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>东北制药</t>
+          <t>中集车辆</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -2569,17 +2569,17 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>603279</t>
+          <t>001338</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>景津装备</t>
+          <t>永顺泰</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -2594,17 +2594,17 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>001338</t>
+          <t>603279</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>永顺泰</t>
+          <t>景津装备</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
@@ -2619,17 +2619,17 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>002390</t>
+          <t>688330</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>信邦制药</t>
+          <t>宏力达</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -2644,17 +2644,17 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>688330</t>
+          <t>002390</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>宏力达</t>
+          <t>信邦制药</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -2744,17 +2744,17 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>601002</t>
+          <t>300389</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>晋亿实业</t>
+          <t>艾比森</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -2769,17 +2769,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>300389</t>
+          <t>002081</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>艾比森</t>
+          <t>金 螳 螂</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -2794,12 +2794,12 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>002081</t>
+          <t>601002</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>金 螳 螂</t>
+          <t>晋亿实业</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">

</xml_diff>

<commit_message>
数据更新 2026-08-29（GitHub Actions 自动）
模式：daily

═══ 数据状态 ═══
  指数: 2026-08-28 ✓
  ETF: 2026-08-28 ✓
  推荐20: 2026-08-28 ✓
  其他成份: 2026-08-28 ✓
  自选: 2026-08-28 ✓
  成分样本: 2026-08-28 ✓
  季度检测: 从未执行（深度更新或维护可执行）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9.32</v>
+        <v>9.359999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9.18</v>
+        <v>9.039999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6.14</v>
+        <v>6.06</v>
       </c>
     </row>
     <row r="5">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5.43</v>
+        <v>5.41</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.18</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="7">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>4.19</v>
+        <v>4.24</v>
       </c>
     </row>
     <row r="8">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>4.13</v>
+        <v>4.09</v>
       </c>
     </row>
     <row r="9">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3.5</v>
+        <v>3.47</v>
       </c>
     </row>
     <row r="10">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3.35</v>
+        <v>3.32</v>
       </c>
     </row>
     <row r="11">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3.13</v>
+        <v>3.19</v>
       </c>
     </row>
     <row r="12">
@@ -869,12 +869,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>600170</t>
+          <t>600057</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>上海建工</t>
+          <t>厦门象屿</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -894,12 +894,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>600057</t>
+          <t>600170</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>厦门象屿</t>
+          <t>上海建工</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1044,17 +1044,17 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>600741</t>
+          <t>000959</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>华域汽车</t>
+          <t>首钢股份</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1094,17 +1094,17 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>000959</t>
+          <t>600741</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>首钢股份</t>
+          <t>华域汽车</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1269,17 +1269,17 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>600398</t>
+          <t>600352</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>海澜之家</t>
+          <t>浙江龙盛</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1294,17 +1294,17 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>600295</t>
+          <t>600398</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>鄂尔多斯</t>
+          <t>海澜之家</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>600352</t>
+          <t>600295</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>浙江龙盛</t>
+          <t>鄂尔多斯</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1669,17 +1669,17 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>600267</t>
+          <t>002761</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>海正药业</t>
+          <t>浙江建投</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -1694,17 +1694,17 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>002761</t>
+          <t>600267</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>浙江建投</t>
+          <t>海正药业</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -1894,17 +1894,17 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>002004</t>
+          <t>601339</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>华邦健康</t>
+          <t>百隆东方</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -1919,17 +1919,17 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>601339</t>
+          <t>002004</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>百隆东方</t>
+          <t>华邦健康</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -1969,12 +1969,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>002061</t>
+          <t>000090</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>浙江交科</t>
+          <t>天健集团</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -1994,12 +1994,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>000090</t>
+          <t>002061</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>天健集团</t>
+          <t>浙江交科</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -2019,17 +2019,17 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>002727</t>
+          <t>002416</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>一心堂</t>
+          <t>爱施德</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -2044,17 +2044,17 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>002416</t>
+          <t>002727</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>爱施德</t>
+          <t>一心堂</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -2094,17 +2094,17 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>002170</t>
+          <t>600163</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>芭田股份</t>
+          <t>中闽能源</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -2119,17 +2119,17 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>600163</t>
+          <t>002170</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>中闽能源</t>
+          <t>芭田股份</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -2369,12 +2369,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>600195</t>
+          <t>600300</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>中牧股份</t>
+          <t>维维股份</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -2394,12 +2394,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>600300</t>
+          <t>600195</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>维维股份</t>
+          <t>中牧股份</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -2544,17 +2544,17 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>605377</t>
+          <t>001338</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>华旺科技</t>
+          <t>永顺泰</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -2569,17 +2569,17 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>001338</t>
+          <t>605377</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>永顺泰</t>
+          <t>华旺科技</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -2619,17 +2619,17 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>688330</t>
+          <t>002390</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>宏力达</t>
+          <t>信邦制药</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -2644,17 +2644,17 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>002390</t>
+          <t>688330</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>信邦制药</t>
+          <t>宏力达</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -2744,17 +2744,17 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>300389</t>
+          <t>002918</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>艾比森</t>
+          <t>蒙娜丽莎</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -2769,12 +2769,12 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>002081</t>
+          <t>601002</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>金 螳 螂</t>
+          <t>晋亿实业</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -2794,17 +2794,17 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>601002</t>
+          <t>300389</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>晋亿实业</t>
+          <t>艾比森</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -2819,17 +2819,17 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>000026</t>
+          <t>002081</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>飞亚达</t>
+          <t>金 螳 螂</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -2869,17 +2869,17 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>002918</t>
+          <t>000026</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>蒙娜丽莎</t>
+          <t>飞亚达</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">

</xml_diff>

<commit_message>
数据更新 2026-08-31（GitHub Actions 自动）
模式：weekly

═══ 数据状态 ═══
  指数: 2026-08-31 ✓
  ETF: 2026-08-31 ✓
  推荐20: 2026-08-31 ✓
  其他成份: 2026-08-31 ✓
  自选: 2026-08-31 ✓
  成分样本: 2026-08-31 ✓
  季度检测: 从未执行（深度更新或维护可执行）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9.359999999999999</v>
+        <v>9.49</v>
       </c>
     </row>
     <row r="3">
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9.039999999999999</v>
+        <v>9.130000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6.06</v>
+        <v>6.05</v>
       </c>
     </row>
     <row r="5">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5.41</v>
+        <v>5.35</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.2</v>
+        <v>5.22</v>
       </c>
     </row>
     <row r="7">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>4.24</v>
+        <v>4.21</v>
       </c>
     </row>
     <row r="8">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>4.09</v>
+        <v>4.19</v>
       </c>
     </row>
     <row r="9">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3.47</v>
+        <v>3.48</v>
       </c>
     </row>
     <row r="10">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3.32</v>
+        <v>3.31</v>
       </c>
     </row>
     <row r="11">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3.19</v>
+        <v>3.13</v>
       </c>
     </row>
     <row r="12">
@@ -819,17 +819,17 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>601117</t>
+          <t>601898</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>中国化学</t>
+          <t>中煤能源</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -844,17 +844,17 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>601898</t>
+          <t>601117</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>中煤能源</t>
+          <t>中国化学</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1219,17 +1219,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>601880</t>
+          <t>000921</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>辽港股份</t>
+          <t>海信家电</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1244,17 +1244,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>000921</t>
+          <t>601880</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>海信家电</t>
+          <t>辽港股份</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1269,12 +1269,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>600352</t>
+          <t>600295</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>浙江龙盛</t>
+          <t>鄂尔多斯</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>600295</t>
+          <t>600352</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>鄂尔多斯</t>
+          <t>浙江龙盛</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1519,17 +1519,17 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>600258</t>
+          <t>601083</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>首旅酒店</t>
+          <t>锦江航运</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -1544,17 +1544,17 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>601083</t>
+          <t>600258</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>锦江航运</t>
+          <t>首旅酒店</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -1619,17 +1619,17 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>000513</t>
+          <t>603766</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>丽珠集团</t>
+          <t>隆鑫通用</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -1644,17 +1644,17 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>603766</t>
+          <t>000513</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>隆鑫通用</t>
+          <t>丽珠集团</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -1744,17 +1744,17 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>000400</t>
+          <t>300244</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>许继电气</t>
+          <t>迪安诊断</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -1769,17 +1769,17 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>300244</t>
+          <t>000400</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>迪安诊断</t>
+          <t>许继电气</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -1794,17 +1794,17 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>002545</t>
+          <t>002039</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>东方铁塔</t>
+          <t>黔源电力</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -1819,17 +1819,17 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>002039</t>
+          <t>002545</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>黔源电力</t>
+          <t>东方铁塔</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -1869,17 +1869,17 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>600004</t>
+          <t>601339</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>白云机场</t>
+          <t>百隆东方</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -1894,17 +1894,17 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>601339</t>
+          <t>600004</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>百隆东方</t>
+          <t>白云机场</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -1969,17 +1969,17 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>000090</t>
+          <t>000719</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>天健集团</t>
+          <t>中原传媒</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -1994,17 +1994,17 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>002061</t>
+          <t>002416</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>浙江交科</t>
+          <t>爱施德</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -2019,17 +2019,17 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>002416</t>
+          <t>000090</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>爱施德</t>
+          <t>天健集团</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -2044,17 +2044,17 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>002727</t>
+          <t>002061</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>一心堂</t>
+          <t>浙江交科</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -2069,17 +2069,17 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>000719</t>
+          <t>002727</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>中原传媒</t>
+          <t>一心堂</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -2094,17 +2094,17 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>600163</t>
+          <t>002170</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>中闽能源</t>
+          <t>芭田股份</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -2119,17 +2119,17 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>002170</t>
+          <t>600163</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>芭田股份</t>
+          <t>中闽能源</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -2369,12 +2369,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>600300</t>
+          <t>600195</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>维维股份</t>
+          <t>中牧股份</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -2394,12 +2394,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>600195</t>
+          <t>600300</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>中牧股份</t>
+          <t>维维股份</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -2519,17 +2519,17 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>601801</t>
+          <t>688330</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>皖新传媒</t>
+          <t>宏力达</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -2544,17 +2544,17 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>001338</t>
+          <t>601801</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>永顺泰</t>
+          <t>皖新传媒</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -2594,17 +2594,17 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>603279</t>
+          <t>001338</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>景津装备</t>
+          <t>永顺泰</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
@@ -2619,17 +2619,17 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>002390</t>
+          <t>603279</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>信邦制药</t>
+          <t>景津装备</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -2644,17 +2644,17 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>688330</t>
+          <t>002390</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>宏力达</t>
+          <t>信邦制药</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -2669,17 +2669,17 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>600351</t>
+          <t>600897</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>亚宝药业</t>
+          <t>厦门空港</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -2694,17 +2694,17 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>600897</t>
+          <t>600351</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>厦门空港</t>
+          <t>亚宝药业</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -2719,17 +2719,17 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>002478</t>
+          <t>002081</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>常宝股份</t>
+          <t>金 螳 螂</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -2744,12 +2744,12 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>002918</t>
+          <t>601002</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>蒙娜丽莎</t>
+          <t>晋亿实业</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -2769,17 +2769,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>601002</t>
+          <t>002478</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>晋亿实业</t>
+          <t>常宝股份</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -2794,17 +2794,17 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>300389</t>
+          <t>002918</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>艾比森</t>
+          <t>蒙娜丽莎</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -2819,17 +2819,17 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>002081</t>
+          <t>300389</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>金 螳 螂</t>
+          <t>艾比森</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -2844,17 +2844,17 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>300228</t>
+          <t>000026</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>富瑞特装</t>
+          <t>飞亚达</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -2869,17 +2869,17 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>000026</t>
+          <t>300228</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>飞亚达</t>
+          <t>富瑞特装</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">

</xml_diff>

<commit_message>
数据更新 2026-09-01（GitHub Actions 自动）
模式：daily

═══ 数据状态 ═══
  指数: 2026-09-01 ✓
  ETF: 2026-09-01 ✓
  推荐20: 2026-09-01 ✓
  其他成份: 2026-09-01 ✓
  自选: 2026-09-01 ✓
  成分样本: 2026-09-01 ✓
  季度检测: 从未执行（深度更新或维护可执行）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9.49</v>
+        <v>9.44</v>
       </c>
     </row>
     <row r="3">
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9.130000000000001</v>
+        <v>9.27</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6.05</v>
+        <v>5.98</v>
       </c>
     </row>
     <row r="5">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5.35</v>
+        <v>5.36</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.22</v>
+        <v>5.27</v>
       </c>
     </row>
     <row r="7">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>4.21</v>
+        <v>4.22</v>
       </c>
     </row>
     <row r="8">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>4.19</v>
+        <v>4.12</v>
       </c>
     </row>
     <row r="9">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3.48</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="10">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3.31</v>
+        <v>3.29</v>
       </c>
     </row>
     <row r="11">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3.13</v>
+        <v>3.15</v>
       </c>
     </row>
     <row r="12">
@@ -819,17 +819,17 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>601898</t>
+          <t>601117</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>中煤能源</t>
+          <t>中国化学</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -844,17 +844,17 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>601117</t>
+          <t>601898</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>中国化学</t>
+          <t>中煤能源</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1069,17 +1069,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>600096</t>
+          <t>600741</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>云天化</t>
+          <t>华域汽车</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1094,17 +1094,17 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>600741</t>
+          <t>600096</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>华域汽车</t>
+          <t>云天化</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1194,17 +1194,17 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>600546</t>
+          <t>000921</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>山煤国际</t>
+          <t>海信家电</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1219,17 +1219,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>000921</t>
+          <t>601880</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>海信家电</t>
+          <t>辽港股份</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1244,17 +1244,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>601880</t>
+          <t>600546</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>辽港股份</t>
+          <t>山煤国际</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1519,17 +1519,17 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>601083</t>
+          <t>600258</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>锦江航运</t>
+          <t>首旅酒店</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -1544,17 +1544,17 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>600258</t>
+          <t>601083</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>首旅酒店</t>
+          <t>锦江航运</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -1594,17 +1594,17 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>601001</t>
+          <t>000513</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>晋控煤业</t>
+          <t>丽珠集团</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -1644,17 +1644,17 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>000513</t>
+          <t>601001</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>丽珠集团</t>
+          <t>晋控煤业</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -1744,17 +1744,17 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>300244</t>
+          <t>000400</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>迪安诊断</t>
+          <t>许继电气</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -1769,17 +1769,17 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>000400</t>
+          <t>300244</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>许继电气</t>
+          <t>迪安诊断</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -1994,17 +1994,17 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>002416</t>
+          <t>000090</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>爱施德</t>
+          <t>天健集团</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -2019,17 +2019,17 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>000090</t>
+          <t>002416</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>天健集团</t>
+          <t>爱施德</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -2044,17 +2044,17 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>002061</t>
+          <t>002727</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>浙江交科</t>
+          <t>一心堂</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -2069,17 +2069,17 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>002727</t>
+          <t>002061</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>一心堂</t>
+          <t>浙江交科</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -2094,17 +2094,17 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>002170</t>
+          <t>600163</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>芭田股份</t>
+          <t>中闽能源</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -2119,17 +2119,17 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>600163</t>
+          <t>002170</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>中闽能源</t>
+          <t>芭田股份</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -2319,17 +2319,17 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>002043</t>
+          <t>603708</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>兔 宝 宝</t>
+          <t>家家悦</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -2344,17 +2344,17 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>603708</t>
+          <t>002043</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>家家悦</t>
+          <t>兔 宝 宝</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -2369,12 +2369,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>600195</t>
+          <t>600300</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>中牧股份</t>
+          <t>维维股份</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -2394,12 +2394,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>600300</t>
+          <t>600195</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>维维股份</t>
+          <t>中牧股份</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -2519,17 +2519,17 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>688330</t>
+          <t>601801</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>宏力达</t>
+          <t>皖新传媒</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -2544,17 +2544,17 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>601801</t>
+          <t>688330</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>皖新传媒</t>
+          <t>宏力达</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -2569,17 +2569,17 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>605377</t>
+          <t>001338</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>华旺科技</t>
+          <t>永顺泰</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -2594,17 +2594,17 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>001338</t>
+          <t>605377</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>永顺泰</t>
+          <t>华旺科技</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
@@ -2719,17 +2719,17 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>002081</t>
+          <t>002478</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>金 螳 螂</t>
+          <t>常宝股份</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -2744,12 +2744,12 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>601002</t>
+          <t>002918</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>晋亿实业</t>
+          <t>蒙娜丽莎</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -2769,17 +2769,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>002478</t>
+          <t>601002</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>常宝股份</t>
+          <t>晋亿实业</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -2794,17 +2794,17 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>002918</t>
+          <t>300389</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>蒙娜丽莎</t>
+          <t>艾比森</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -2819,17 +2819,17 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>300389</t>
+          <t>002081</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>艾比森</t>
+          <t>金 螳 螂</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">

</xml_diff>

<commit_message>
数据更新 2026-09-07（GitHub Actions 自动）
模式：weekly

═══ 数据状态 ═══
  指数: 2026-09-07 ✓
  ETF: 2026-09-07 ✓
  推荐20: 2026-09-07 ✓
  其他成份: 2026-09-07 ✓
  自选: 2026-09-07 ✓
  成分样本: 2026-09-07 ✓
  季度检测: 从未执行（深度更新或维护可执行）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="980092" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="980092" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'980092'!$A$1:$E$101</definedName>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9.23</v>
+        <v>9.210000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9.220000000000001</v>
+        <v>9.18</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6.1</v>
+        <v>6.12</v>
       </c>
     </row>
     <row r="5">
@@ -558,12 +558,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>601633</t>
+          <t>600104</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>长城汽车</t>
+          <t>上汽集团</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5.31</v>
+        <v>5.38</v>
       </c>
     </row>
     <row r="6">
@@ -581,12 +581,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>600104</t>
+          <t>601633</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>上汽集团</t>
+          <t>长城汽车</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.31</v>
+        <v>5.34</v>
       </c>
     </row>
     <row r="7">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>4.21</v>
+        <v>4.17</v>
       </c>
     </row>
     <row r="8">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>3.99</v>
+        <v>4.01</v>
       </c>
     </row>
     <row r="9">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3.47</v>
+        <v>3.46</v>
       </c>
     </row>
     <row r="10">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3.12</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="12">
@@ -1044,17 +1044,17 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>000959</t>
+          <t>600741</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>首钢股份</t>
+          <t>华域汽车</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1069,17 +1069,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>600741</t>
+          <t>000959</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>华域汽车</t>
+          <t>首钢股份</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1244,17 +1244,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>600295</t>
+          <t>600546</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>鄂尔多斯</t>
+          <t>山煤国际</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1269,17 +1269,17 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>600546</t>
+          <t>600295</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>山煤国际</t>
+          <t>鄂尔多斯</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1319,17 +1319,17 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>600352</t>
+          <t>603444</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>浙江龙盛</t>
+          <t>吉比特</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1344,17 +1344,17 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>600060</t>
+          <t>600352</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>海信视像</t>
+          <t>浙江龙盛</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -1369,17 +1369,17 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>688819</t>
+          <t>600060</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>天能股份</t>
+          <t>海信视像</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -1394,17 +1394,17 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>603444</t>
+          <t>688819</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>吉比特</t>
+          <t>天能股份</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -1794,17 +1794,17 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>002039</t>
+          <t>600729</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>黔源电力</t>
+          <t>重百集团</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -1819,17 +1819,17 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>002545</t>
+          <t>002039</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>东方铁塔</t>
+          <t>黔源电力</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -1844,17 +1844,17 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>600729</t>
+          <t>600004</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>重百集团</t>
+          <t>白云机场</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -1869,17 +1869,17 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>600004</t>
+          <t>002545</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>白云机场</t>
+          <t>东方铁塔</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -1919,17 +1919,17 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>000957</t>
+          <t>002004</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>中通客车</t>
+          <t>华邦健康</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -1944,17 +1944,17 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>002004</t>
+          <t>000957</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>华邦健康</t>
+          <t>中通客车</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -2019,17 +2019,17 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>002727</t>
+          <t>000090</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>一心堂</t>
+          <t>天健集团</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -2044,17 +2044,17 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>000090</t>
+          <t>002727</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>天健集团</t>
+          <t>一心堂</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -2219,17 +2219,17 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>000597</t>
+          <t>002697</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>东北制药</t>
+          <t>红旗连锁</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -2244,17 +2244,17 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>301039</t>
+          <t>000597</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>中集车辆</t>
+          <t>东北制药</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -2269,17 +2269,17 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>002697</t>
+          <t>301039</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>红旗连锁</t>
+          <t>中集车辆</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -2319,17 +2319,17 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>002043</t>
+          <t>603708</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>兔 宝 宝</t>
+          <t>家家悦</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -2344,12 +2344,12 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>603708</t>
+          <t>600195</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>家家悦</t>
+          <t>中牧股份</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -2369,12 +2369,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>600195</t>
+          <t>600300</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>中牧股份</t>
+          <t>维维股份</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -2394,17 +2394,17 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>600300</t>
+          <t>002043</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>维维股份</t>
+          <t>兔 宝 宝</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -2494,17 +2494,17 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>000650</t>
+          <t>601801</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>仁和药业</t>
+          <t>皖新传媒</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -2519,17 +2519,17 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>601801</t>
+          <t>000650</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>皖新传媒</t>
+          <t>仁和药业</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -2544,17 +2544,17 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>688330</t>
+          <t>001338</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>宏力达</t>
+          <t>永顺泰</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>主要消费</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -2569,17 +2569,17 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>001338</t>
+          <t>688330</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>永顺泰</t>
+          <t>宏力达</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>主要消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -2769,17 +2769,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>300389</t>
+          <t>000026</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>艾比森</t>
+          <t>飞亚达</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -2794,17 +2794,17 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>002918</t>
+          <t>300389</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>蒙娜丽莎</t>
+          <t>艾比森</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -2819,17 +2819,17 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>000026</t>
+          <t>002918</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>飞亚达</t>
+          <t>蒙娜丽莎</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">

</xml_diff>

<commit_message>
数据更新 2026-09-08（GitHub Actions 自动）
模式：daily

═══ 数据状态 ═══
  指数: 2026-09-08 ✓
  ETF: 2026-09-08 ✓
  推荐20: 2026-09-08 ✓
  其他成份: 2026-09-08 ✓
  自选: 2026-09-08 ✓
  成分样本: 2026-09-08 ✓
  季度检测: 从未执行（深度更新或维护可执行）
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -489,21 +489,21 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>601728</t>
+          <t>600938</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>中国电信</t>
+          <t>中国海油</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>电信业务</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>9.210000000000001</v>
+        <v>9.460000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -512,21 +512,21 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>600938</t>
+          <t>601728</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>中国海油</t>
+          <t>中国电信</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>电信业务</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9.18</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6.12</v>
+        <v>5.98</v>
       </c>
     </row>
     <row r="5">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5.38</v>
+        <v>5.41</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.34</v>
+        <v>5.33</v>
       </c>
     </row>
     <row r="7">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>4.17</v>
+        <v>4.22</v>
       </c>
     </row>
     <row r="8">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>4.01</v>
+        <v>3.94</v>
       </c>
     </row>
     <row r="9">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3.46</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="10">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3.37</v>
+        <v>3.31</v>
       </c>
     </row>
     <row r="11">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3.21</v>
+        <v>3.08</v>
       </c>
     </row>
     <row r="12">
@@ -869,12 +869,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>600057</t>
+          <t>600170</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>厦门象屿</t>
+          <t>上海建工</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -894,12 +894,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>600170</t>
+          <t>600057</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>上海建工</t>
+          <t>厦门象屿</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1044,17 +1044,17 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>600741</t>
+          <t>000959</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>华域汽车</t>
+          <t>首钢股份</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1069,12 +1069,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>000959</t>
+          <t>600096</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>首钢股份</t>
+          <t>云天化</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1094,17 +1094,17 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>600096</t>
+          <t>600741</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>云天化</t>
+          <t>华域汽车</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1119,17 +1119,17 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>601156</t>
+          <t>600256</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>东航物流</t>
+          <t>广汇能源</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>能源</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1144,17 +1144,17 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>600256</t>
+          <t>601156</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>广汇能源</t>
+          <t>东航物流</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>能源</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1319,17 +1319,17 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>603444</t>
+          <t>600352</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>吉比特</t>
+          <t>浙江龙盛</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1344,17 +1344,17 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>600352</t>
+          <t>603444</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>浙江龙盛</t>
+          <t>吉比特</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -1369,17 +1369,17 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>600060</t>
+          <t>688819</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>海信视像</t>
+          <t>天能股份</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -1394,17 +1394,17 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>688819</t>
+          <t>600060</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>天能股份</t>
+          <t>海信视像</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -1544,17 +1544,17 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>601083</t>
+          <t>600874</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>锦江航运</t>
+          <t>创业环保</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -1569,17 +1569,17 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>600874</t>
+          <t>601083</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>创业环保</t>
+          <t>锦江航运</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -1819,17 +1819,17 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>002039</t>
+          <t>002545</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>黔源电力</t>
+          <t>东方铁塔</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>公用事业</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -1844,17 +1844,17 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>600004</t>
+          <t>002039</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>白云机场</t>
+          <t>黔源电力</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>公用事业</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -1869,17 +1869,17 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>002545</t>
+          <t>600004</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>东方铁塔</t>
+          <t>白云机场</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -1894,17 +1894,17 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>601339</t>
+          <t>002004</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>百隆东方</t>
+          <t>华邦健康</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>原材料</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -1919,17 +1919,17 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>002004</t>
+          <t>000957</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>华邦健康</t>
+          <t>中通客车</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -1944,12 +1944,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>000957</t>
+          <t>601339</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>中通客车</t>
+          <t>百隆东方</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -1994,17 +1994,17 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>002416</t>
+          <t>000090</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>爱施德</t>
+          <t>天健集团</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -2019,17 +2019,17 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>000090</t>
+          <t>002416</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>天健集团</t>
+          <t>爱施德</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -2269,17 +2269,17 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>301039</t>
+          <t>000915</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>中集车辆</t>
+          <t>华特达因</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -2294,17 +2294,17 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>000915</t>
+          <t>301039</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>华特达因</t>
+          <t>中集车辆</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
@@ -2444,17 +2444,17 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>603368</t>
+          <t>603173</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>柳药集团</t>
+          <t>福斯达</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -2469,17 +2469,17 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>603173</t>
+          <t>603368</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>福斯达</t>
+          <t>柳药集团</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -2644,17 +2644,17 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>600897</t>
+          <t>002390</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>厦门空港</t>
+          <t>信邦制药</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>医药卫生</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -2669,17 +2669,17 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>002390</t>
+          <t>600897</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>信邦制药</t>
+          <t>厦门空港</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>医药卫生</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -2769,17 +2769,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>000026</t>
+          <t>300389</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>飞亚达</t>
+          <t>艾比森</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>可选消费</t>
+          <t>信息技术</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -2794,17 +2794,17 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>300389</t>
+          <t>002918</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>艾比森</t>
+          <t>蒙娜丽莎</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>信息技术</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -2819,12 +2819,12 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>002918</t>
+          <t>002081</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>蒙娜丽莎</t>
+          <t>金 螳 螂</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -2844,17 +2844,17 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>002081</t>
+          <t>000026</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>金 螳 螂</t>
+          <t>飞亚达</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>工业</t>
+          <t>可选消费</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">

</xml_diff>

<commit_message>
manifest 增加 per-标的 ind_last/stale 陈旧标记（T3）
- 根因：manifest 只有全局 data_date，单只标的指标冻结被掩盖（920599 曾冻结 10 个交易日而 manifest 全绿）

- 修复：build_manifest 复用已解析的指标文件末行日期 → 每标的 ind_last（零额外 IO）；落后 data_date >=3 自然日 → stale=true；顶层加 stale_n；存在陈旧项时打印告警

- 阈值 STALE_LAG_DAYS 收进 _common.py，与 update.py status 清单共用（单一来源）

- 验证：manifest 364/364 有 ind_last、stale_n=1（仅 920599）、analysis.date==data_date；_test_analysis.py --no-snapshot 60/60 PASS

- 数据漂移：update.py web 顺带重拉 ETF 季报持仓，980092/159201 估算 dy 3.1854→3.1801（-0.17%），推荐20 成员与分数不变
</commit_message>
<xml_diff>
--- a/excel/国证指数成分.xlsx
+++ b/excel/国证指数成分.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="980092" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="980092" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'980092'!$A$1:$E$101</definedName>

</xml_diff>